<commit_message>
Feat: Reécriture intégrale de tous les conseils de l Excel en phrases complètes, claires et explicatives
</commit_message>
<xml_diff>
--- a/config/rules/tableau_oria.xlsx
+++ b/config/rules/tableau_oria.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ou Urgences 15</t>
+          <t>En cas de danger immédiat ou de détresse vitale, composer directement le 15 (SAMU), le 17 (Police/Gendarmerie) ou le 112.</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3919 violences faites aux femmes</t>
+          <t>Orientation d'urgence vers le 3919 (Violences Femmes Info, numéro gratuit et anonyme 24h/24).</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARS/CD +3977+ ou appeler de service</t>
+          <t>Contacter le 3977 (Plateforme contre les maltraitances envers les personnes âgées) et effectuer un signalement auprès de l'ARS et du Conseil Départemental.</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       <c r="U10" s="5" t="n"/>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>POLICE + ARS/CD + 3977</t>
+          <t>Effectuer un signalement auprès du 3977 (lutte contre les maltraitances) ainsi qu'auprès des services de l'ARS, du Conseil Départemental et des forces de l'ordre.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       <c r="U14" s="5" t="n"/>
       <c r="V14" s="4" t="inlineStr">
         <is>
-          <t>Médicalib + asso kiné</t>
+          <t>Consulter des plateformes de mise en relation comme Libheros ou Médicalib, et se rapprocher de l'association locale de masso-kinésithérapie.</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       <c r="U16" s="4" t="n"/>
       <c r="V16" s="4" t="inlineStr">
         <is>
-          <t>Médicalib + asso d'IDEL</t>
+          <t>Rechercher un infirmier libéral qualifié via Médicalib, Libheros ou l'annuaire de l'Ordre National des Infirmiers.</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       <c r="U23" s="5" t="n"/>
       <c r="V23" s="4" t="inlineStr">
         <is>
-          <t>Contacter services d'aides à dom</t>
+          <t>Solliciter et comparer les services d'aide et d'accompagnement à domicile (SAAD) agréés du secteur pour la mise en place d'intervenants qualifiés.</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       <c r="U31" s="4" t="n"/>
       <c r="V31" s="4" t="inlineStr">
         <is>
-          <t>Asso des aidants</t>
+          <t>Proposer des solutions de répit en orientant l'aidant vers l'Association Française des Aidants, la Plateforme d'Accompagnement et de Répit (PFR) locale ou le Café des Aidants.</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
       <c r="U38" s="4" t="n"/>
       <c r="V38" s="4" t="inlineStr">
         <is>
-          <t>orientation vers médecin traitant ou spécialiste</t>
+          <t>Prendre rendez-vous en priorité auprès du médecin traitant pour planifier une consultation gériatrique ou une orientation vers un médecin spécialiste.</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
       <c r="U57" s="4" t="n"/>
       <c r="V57" s="4" t="inlineStr">
         <is>
-          <t>Sociétés de nettoyage</t>
+          <t>Faire appel à des sociétés spécialisées dans le nettoyage extrême et la désinfection de logements insalubres (syndrome de Diogène) en lien avec le service communale d'hygiène et de santé (SCHS).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Retrait de Libheros et alignement strict sur les notes originales de l Excel
</commit_message>
<xml_diff>
--- a/config/rules/tableau_oria.xlsx
+++ b/config/rules/tableau_oria.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>En cas de danger immédiat ou de détresse vitale, composer directement le 15 (SAMU), le 17 (Police/Gendarmerie) ou le 112.</t>
+          <t>Ou Urgences 15</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Orientation d'urgence vers le 3919 (Violences Femmes Info, numéro gratuit et anonyme 24h/24).</t>
+          <t>3919 violences faites aux femmes</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Contacter le 3977 (Plateforme contre les maltraitances envers les personnes âgées) et effectuer un signalement auprès de l'ARS et du Conseil Départemental.</t>
+          <t>ARS/CD + 3977 ou appeler de service</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       <c r="U10" s="5" t="n"/>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>Effectuer un signalement auprès du 3977 (lutte contre les maltraitances) ainsi qu'auprès des services de l'ARS, du Conseil Départemental et des forces de l'ordre.</t>
+          <t>POLICE + ARS/CD + 3977</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       <c r="U14" s="5" t="n"/>
       <c r="V14" s="4" t="inlineStr">
         <is>
-          <t>Consulter des plateformes de mise en relation comme Libheros ou Médicalib, et se rapprocher de l'association locale de masso-kinésithérapie.</t>
+          <t>Médicalib + association de kinésithérapie</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       <c r="U16" s="4" t="n"/>
       <c r="V16" s="4" t="inlineStr">
         <is>
-          <t>Rechercher un infirmier libéral qualifié via Médicalib, Libheros ou l'annuaire de l'Ordre National des Infirmiers.</t>
+          <t>Médicalib + association d'IDEL</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       <c r="U23" s="5" t="n"/>
       <c r="V23" s="4" t="inlineStr">
         <is>
-          <t>Solliciter et comparer les services d'aide et d'accompagnement à domicile (SAAD) agréés du secteur pour la mise en place d'intervenants qualifiés.</t>
+          <t>Contacter les services d'aide à domicile</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       <c r="U31" s="4" t="n"/>
       <c r="V31" s="4" t="inlineStr">
         <is>
-          <t>Proposer des solutions de répit en orientant l'aidant vers l'Association Française des Aidants, la Plateforme d'Accompagnement et de Répit (PFR) locale ou le Café des Aidants.</t>
+          <t>Association des aidants</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
       <c r="U38" s="4" t="n"/>
       <c r="V38" s="4" t="inlineStr">
         <is>
-          <t>Prendre rendez-vous en priorité auprès du médecin traitant pour planifier une consultation gériatrique ou une orientation vers un médecin spécialiste.</t>
+          <t>Orientation vers le médecin traitant ou un spécialiste</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
       <c r="U57" s="4" t="n"/>
       <c r="V57" s="4" t="inlineStr">
         <is>
-          <t>Faire appel à des sociétés spécialisées dans le nettoyage extrême et la désinfection de logements insalubres (syndrome de Diogène) en lien avec le service communale d'hygiène et de santé (SCHS).</t>
+          <t>Sociétés de nettoyage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Reformulation des conseils en phrases fluides strictement basees sur les notes originales de l Excel
</commit_message>
<xml_diff>
--- a/config/rules/tableau_oria.xlsx
+++ b/config/rules/tableau_oria.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ou Urgences 15</t>
+          <t>Contacter les Urgences au 15.</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3919 violences faites aux femmes</t>
+          <t>Contacter le 3919 pour les violences faites aux femmes.</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARS/CD + 3977 ou appeler de service</t>
+          <t>Contacter l'ARS/CD et le 3977 ou appeler le service concerné.</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       <c r="U10" s="5" t="n"/>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>POLICE + ARS/CD + 3977</t>
+          <t>Effectuer un signalement auprès du 3977, de l'ARS/CD et des services de Police.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       <c r="U14" s="5" t="n"/>
       <c r="V14" s="4" t="inlineStr">
         <is>
-          <t>Médicalib + association de kinésithérapie</t>
+          <t>Consulter Médicalib ou se rapprocher de l'association de kinésithérapie.</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       <c r="U16" s="4" t="n"/>
       <c r="V16" s="4" t="inlineStr">
         <is>
-          <t>Médicalib + association d'IDEL</t>
+          <t>Consulter Médicalib ou se rapprocher de l'association d'infirmiers (IDEL).</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       <c r="U23" s="5" t="n"/>
       <c r="V23" s="4" t="inlineStr">
         <is>
-          <t>Contacter les services d'aide à domicile</t>
+          <t>Contacter les services d'aide à domicile du secteur.</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       <c r="U31" s="4" t="n"/>
       <c r="V31" s="4" t="inlineStr">
         <is>
-          <t>Association des aidants</t>
+          <t>Se rapprocher de l'association des aidants.</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
       <c r="U38" s="4" t="n"/>
       <c r="V38" s="4" t="inlineStr">
         <is>
-          <t>Orientation vers le médecin traitant ou un spécialiste</t>
+          <t>S'orienter vers le médecin traitant ou un médecin spécialiste.</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
       <c r="U57" s="4" t="n"/>
       <c r="V57" s="4" t="inlineStr">
         <is>
-          <t>Sociétés de nettoyage</t>
+          <t>Faire appel à des sociétés de nettoyage.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Ajout des liens cliquables dans les conseils pour Medicalib, SSIAD, SAAD, Ma Boussole Aidants et Nettoyage Diogene Var
</commit_message>
<xml_diff>
--- a/config/rules/tableau_oria.xlsx
+++ b/config/rules/tableau_oria.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="16608" windowHeight="8712" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="01_Critère_prio_exclu" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="02_Besoins_x_structures (2)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -117,13 +117,26 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="1"/>
@@ -259,21 +272,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau6" displayName="Tableau6" ref="A1:E24" headerRowCount="1" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau6" displayName="Tableau6" ref="A1:E24" headerRowCount="1" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:E24"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Catégorie" dataDxfId="7"/>
-    <tableColumn id="2" name="Critère détaillé" dataDxfId="6"/>
-    <tableColumn id="3" name="Action" dataDxfId="5"/>
-    <tableColumn id="4" name="Structure" dataDxfId="4"/>
-    <tableColumn id="5" name="Conseils" dataDxfId="3"/>
+    <tableColumn id="1" name="Catégorie" dataDxfId="8"/>
+    <tableColumn id="2" name="Critère détaillé" dataDxfId="7"/>
+    <tableColumn id="3" name="Action" dataDxfId="6"/>
+    <tableColumn id="4" name="Structure" dataDxfId="5"/>
+    <tableColumn id="5" name="Conseils" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_Besoins_Structures8" displayName="Table_Besoins_Structures8" ref="A1:V57" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_Besoins_Structures8" displayName="Table_Besoins_Structures8" ref="A1:V59" headerRowCount="1">
   <tableColumns count="22">
     <tableColumn id="1" name="Catégorie"/>
     <tableColumn id="2" name="Besoin détaillé"/>
@@ -292,11 +305,11 @@
     <tableColumn id="16" name="CCAS"/>
     <tableColumn id="17" name="COMPAGNONS_BATISSEURS"/>
     <tableColumn id="18" name="PSCG_SS_APA"/>
-    <tableColumn id="19" name="PRADO" dataDxfId="14" dataCellStyle="Normal 2"/>
-    <tableColumn id="21" name="MISAS" dataDxfId="13" dataCellStyle="Normal 2"/>
-    <tableColumn id="22" name="fil d'argent" dataDxfId="12" dataCellStyle="Normal 2"/>
-    <tableColumn id="20" name="CONSULTATION MÉMOIRE" dataDxfId="11" dataCellStyle="Normal 2"/>
-    <tableColumn id="7" name="Conseils" dataDxfId="10" dataCellStyle="Normal 2"/>
+    <tableColumn id="19" name="PRADO" dataDxfId="15" dataCellStyle="Normal 2"/>
+    <tableColumn id="21" name="MISAS" dataDxfId="14" dataCellStyle="Normal 2"/>
+    <tableColumn id="22" name="fil d'argent" dataDxfId="13" dataCellStyle="Normal 2"/>
+    <tableColumn id="20" name="CONSULTATION MÉMOIRE" dataDxfId="12" dataCellStyle="Normal 2"/>
+    <tableColumn id="7" name="Conseils" dataDxfId="11" dataCellStyle="Normal 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -456,13 +469,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col width="28.08203125" customWidth="1" style="11" min="1" max="1"/>
-    <col width="122.83203125" bestFit="1" customWidth="1" style="11" min="2" max="2"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="11" min="3" max="3"/>
-    <col width="26.9140625" bestFit="1" customWidth="1" style="11" min="4" max="4"/>
-    <col width="33.08203125" customWidth="1" style="11" min="5" max="5"/>
+    <col width="28.09765625" customWidth="1" min="1" max="1"/>
+    <col width="122.796875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="26.8984375" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="33.09765625" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -771,7 +784,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="11">
+    <row r="14" ht="18" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>Hospitalisation / sortie</t>
@@ -1015,10 +1028,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" priority="1" operator="containsText" dxfId="2" text="Exclu">
+    <cfRule type="containsText" priority="1" operator="containsText" dxfId="3" text="Exclu">
       <formula>NOT(ISERROR(SEARCH("Exclu",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="2" operator="containsText" dxfId="1" text="Prioritaire">
+    <cfRule type="containsText" priority="2" operator="containsText" dxfId="2" text="Prioritaire">
       <formula>NOT(ISERROR(SEARCH("Prioritaire",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1036,7 +1049,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AB59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.69921875" defaultRowHeight="13.8"/>
   <cols>
     <col width="22" customWidth="1" style="1" min="1" max="1"/>
     <col width="42" customWidth="1" style="1" min="2" max="2"/>
@@ -1044,11 +1057,12 @@
     <col width="15" customWidth="1" style="1" min="4" max="4"/>
     <col width="20" customWidth="1" style="1" min="5" max="6"/>
     <col width="16" customWidth="1" style="1" min="7" max="21"/>
-    <col width="32.08203125" customWidth="1" style="1" min="22" max="22"/>
-    <col width="8.6640625" customWidth="1" style="1" min="23" max="16384"/>
+    <col width="48.09765625" bestFit="1" customWidth="1" style="1" min="22" max="22"/>
+    <col width="8.69921875" customWidth="1" style="1" min="23" max="23"/>
+    <col width="8.69921875" customWidth="1" style="1" min="24" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="11">
+    <row r="1" ht="28.05" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Catégorie</t>
@@ -1166,7 +1180,7 @@
       <c r="AA1" s="6" t="n"/>
       <c r="AB1" s="6" t="n"/>
     </row>
-    <row r="2" ht="28" customHeight="1" s="11">
+    <row r="2" ht="28.05" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1212,9 +1226,9 @@
       <c r="S2" s="5" t="n"/>
       <c r="T2" s="5" t="n"/>
       <c r="U2" s="5" t="n"/>
-      <c r="V2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="17.65" customHeight="1" s="11">
+      <c r="V2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="17.7" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1241,28 +1255,32 @@
         </is>
       </c>
       <c r="F3" s="3" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
-      <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4" t="n"/>
-      <c r="O3" s="4" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="4" t="n"/>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
-      <c r="U3" s="4" t="n"/>
-      <c r="V3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="17.65" customHeight="1" s="11">
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="n"/>
+      <c r="I3" s="11" t="n"/>
+      <c r="J3" s="11" t="n"/>
+      <c r="K3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
+      <c r="N3" s="11" t="n"/>
+      <c r="O3" s="11" t="n"/>
+      <c r="P3" s="11" t="n"/>
+      <c r="Q3" s="11" t="n"/>
+      <c r="R3" s="11" t="n"/>
+      <c r="S3" s="11" t="n"/>
+      <c r="T3" s="11" t="n"/>
+      <c r="U3" s="11" t="n"/>
+      <c r="V3" s="11" t="inlineStr">
+        <is>
+          <t>Contacter le 3919 pour les violences faites aux femmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.7" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1308,9 +1326,13 @@
       <c r="S4" s="5" t="n"/>
       <c r="T4" s="5" t="n"/>
       <c r="U4" s="5" t="n"/>
-      <c r="V4" s="4" t="n"/>
-    </row>
-    <row r="5" ht="17.65" customHeight="1" s="11">
+      <c r="V4" s="11" t="inlineStr">
+        <is>
+          <t>Contacter le 3919 pour les violences faites aux femmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.7" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1337,28 +1359,28 @@
         </is>
       </c>
       <c r="F5" s="3" t="n"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
-      <c r="N5" s="4" t="n"/>
-      <c r="O5" s="4" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="4" t="n"/>
-      <c r="S5" s="4" t="n"/>
-      <c r="T5" s="4" t="n"/>
-      <c r="U5" s="4" t="n"/>
-      <c r="V5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="17.65" customHeight="1" s="11">
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="n"/>
+      <c r="I5" s="11" t="n"/>
+      <c r="J5" s="11" t="n"/>
+      <c r="K5" s="11" t="n"/>
+      <c r="L5" s="11" t="n"/>
+      <c r="M5" s="11" t="n"/>
+      <c r="N5" s="11" t="n"/>
+      <c r="O5" s="11" t="n"/>
+      <c r="P5" s="11" t="n"/>
+      <c r="Q5" s="11" t="n"/>
+      <c r="R5" s="11" t="n"/>
+      <c r="S5" s="11" t="n"/>
+      <c r="T5" s="11" t="n"/>
+      <c r="U5" s="11" t="n"/>
+      <c r="V5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="17.7" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1408,9 +1430,9 @@
       <c r="S6" s="5" t="n"/>
       <c r="T6" s="5" t="n"/>
       <c r="U6" s="5" t="n"/>
-      <c r="V6" s="4" t="n"/>
-    </row>
-    <row r="7" ht="17.65" customHeight="1" s="11">
+      <c r="V6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="17.7" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1437,28 +1459,28 @@
         </is>
       </c>
       <c r="F7" s="3" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="n"/>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="4" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="4" t="n"/>
-      <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
-      <c r="U7" s="4" t="n"/>
-      <c r="V7" s="4" t="n"/>
-    </row>
-    <row r="8" ht="17.65" customHeight="1" s="11">
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="n"/>
+      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
+      <c r="Q7" s="11" t="n"/>
+      <c r="R7" s="11" t="n"/>
+      <c r="S7" s="11" t="n"/>
+      <c r="T7" s="11" t="n"/>
+      <c r="U7" s="11" t="n"/>
+      <c r="V7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="17.7" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1504,9 +1526,9 @@
       <c r="S8" s="5" t="n"/>
       <c r="T8" s="5" t="n"/>
       <c r="U8" s="5" t="n"/>
-      <c r="V8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="17.65" customHeight="1" s="11">
+      <c r="V8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="17.7" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1533,32 +1555,32 @@
         </is>
       </c>
       <c r="F9" s="3" t="n"/>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="n"/>
-      <c r="L9" s="4" t="n"/>
-      <c r="M9" s="4" t="n"/>
-      <c r="N9" s="4" t="n"/>
-      <c r="O9" s="4" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="4" t="n"/>
-      <c r="R9" s="4" t="n"/>
-      <c r="S9" s="4" t="n"/>
-      <c r="T9" s="4" t="n"/>
-      <c r="U9" s="4" t="n"/>
-      <c r="V9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="17.65" customHeight="1" s="11">
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
+      <c r="N9" s="11" t="n"/>
+      <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
+      <c r="Q9" s="11" t="n"/>
+      <c r="R9" s="11" t="n"/>
+      <c r="S9" s="11" t="n"/>
+      <c r="T9" s="11" t="n"/>
+      <c r="U9" s="11" t="n"/>
+      <c r="V9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="55.2" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1604,13 +1626,13 @@
       <c r="S10" s="5" t="n"/>
       <c r="T10" s="5" t="n"/>
       <c r="U10" s="5" t="n"/>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>Effectuer un signalement auprès du 3977, de l'ARS/CD et des services de Police.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1" s="11">
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>Effectuer un signalement auprès du 3977, de l'ARS, du Conseil Départemental et des services de Police.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Urgence / danger</t>
@@ -1637,28 +1659,28 @@
         </is>
       </c>
       <c r="F11" s="3" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
-      <c r="K11" s="4" t="n"/>
-      <c r="L11" s="4" t="n"/>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="n"/>
-      <c r="O11" s="4" t="n"/>
-      <c r="P11" s="4" t="n"/>
-      <c r="Q11" s="4" t="n"/>
-      <c r="R11" s="4" t="n"/>
-      <c r="S11" s="4" t="n"/>
-      <c r="T11" s="4" t="n"/>
-      <c r="U11" s="4" t="n"/>
-      <c r="V11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="17.65" customHeight="1" s="11">
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="n"/>
+      <c r="O11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
+      <c r="Q11" s="11" t="n"/>
+      <c r="R11" s="11" t="n"/>
+      <c r="S11" s="11" t="n"/>
+      <c r="T11" s="11" t="n"/>
+      <c r="U11" s="11" t="n"/>
+      <c r="V11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="17.7" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Santé / accès aux soins</t>
@@ -1708,7 +1730,7 @@
       </c>
       <c r="T12" s="5" t="n"/>
       <c r="U12" s="5" t="n"/>
-      <c r="V12" s="4" t="n"/>
+      <c r="V12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1737,28 +1759,28 @@
         </is>
       </c>
       <c r="F13" s="3" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
-      <c r="L13" s="4" t="n"/>
-      <c r="M13" s="4" t="n"/>
-      <c r="N13" s="4" t="n"/>
-      <c r="O13" s="4" t="n"/>
-      <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="4" t="n"/>
-      <c r="R13" s="4" t="n"/>
-      <c r="S13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T13" s="4" t="n"/>
-      <c r="U13" s="4" t="n"/>
-      <c r="V13" s="4" t="n"/>
-    </row>
-    <row r="14">
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="11" t="n"/>
+      <c r="L13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
+      <c r="N13" s="11" t="n"/>
+      <c r="O13" s="11" t="n"/>
+      <c r="P13" s="11" t="n"/>
+      <c r="Q13" s="11" t="n"/>
+      <c r="R13" s="11" t="n"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="n"/>
+      <c r="U13" s="11" t="n"/>
+      <c r="V13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="27.6" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Santé / accès aux soins</t>
@@ -1808,9 +1830,9 @@
       </c>
       <c r="T14" s="5" t="n"/>
       <c r="U14" s="5" t="n"/>
-      <c r="V14" s="4" t="inlineStr">
-        <is>
-          <t>Consulter Médicalib ou se rapprocher de l'association de kinésithérapie.</t>
+      <c r="V14" s="11" t="inlineStr">
+        <is>
+          <t>Consulter [Medicalib](https://www.medicalib.fr/) ou se rapprocher des associations de kinésithérapie.</t>
         </is>
       </c>
     </row>
@@ -1844,17 +1866,17 @@
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5" t="n"/>
       <c r="Q15" s="5" t="n"/>
-      <c r="R15" s="4" t="n"/>
-      <c r="S15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T15" s="4" t="n"/>
-      <c r="U15" s="4" t="n"/>
-      <c r="V15" s="4" t="n"/>
-    </row>
-    <row r="16">
+      <c r="R15" s="11" t="n"/>
+      <c r="S15" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="n"/>
+      <c r="U15" s="11" t="n"/>
+      <c r="V15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="27.6" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Santé / accès aux soins</t>
@@ -1881,32 +1903,32 @@
         </is>
       </c>
       <c r="F16" s="3" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="n"/>
-      <c r="L16" s="4" t="n"/>
-      <c r="M16" s="4" t="n"/>
-      <c r="N16" s="4" t="n"/>
-      <c r="O16" s="4" t="n"/>
-      <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="4" t="n"/>
-      <c r="R16" s="4" t="n"/>
-      <c r="S16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T16" s="4" t="n"/>
-      <c r="U16" s="4" t="n"/>
-      <c r="V16" s="4" t="inlineStr">
-        <is>
-          <t>Consulter Médicalib ou se rapprocher de l'association d'infirmiers (IDEL).</t>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="11" t="n"/>
+      <c r="I16" s="11" t="n"/>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="11" t="n"/>
+      <c r="M16" s="11" t="n"/>
+      <c r="N16" s="11" t="n"/>
+      <c r="O16" s="11" t="n"/>
+      <c r="P16" s="11" t="n"/>
+      <c r="Q16" s="11" t="n"/>
+      <c r="R16" s="11" t="n"/>
+      <c r="S16" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T16" s="11" t="n"/>
+      <c r="U16" s="11" t="n"/>
+      <c r="V16" s="11" t="inlineStr">
+        <is>
+          <t>Consulter [Medicalib](https://www.medicalib.fr/) ou se rapprocher des associations d'infirmiers (IDEL).</t>
         </is>
       </c>
     </row>
@@ -1952,9 +1974,9 @@
       <c r="S17" s="5" t="n"/>
       <c r="T17" s="5" t="n"/>
       <c r="U17" s="5" t="n"/>
-      <c r="V17" s="4" t="n"/>
-    </row>
-    <row r="18" ht="17.65" customHeight="1" s="11">
+      <c r="V17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="17.7" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Santé / accès aux soins</t>
@@ -1981,28 +2003,28 @@
         </is>
       </c>
       <c r="F18" s="3" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
-      <c r="N18" s="4" t="n"/>
-      <c r="O18" s="4" t="n"/>
-      <c r="P18" s="4" t="n"/>
-      <c r="Q18" s="4" t="n"/>
-      <c r="R18" s="4" t="n"/>
-      <c r="S18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T18" s="4" t="n"/>
-      <c r="U18" s="4" t="n"/>
-      <c r="V18" s="4" t="n"/>
-    </row>
-    <row r="19" ht="17.65" customHeight="1" s="11">
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="11" t="n"/>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="N18" s="11" t="n"/>
+      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="n"/>
+      <c r="Q18" s="11" t="n"/>
+      <c r="R18" s="11" t="n"/>
+      <c r="S18" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T18" s="11" t="n"/>
+      <c r="U18" s="11" t="n"/>
+      <c r="V18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="17.7" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Santé / accès aux soins</t>
@@ -2029,28 +2051,28 @@
         </is>
       </c>
       <c r="F19" s="3" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4" t="n"/>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="4" t="n"/>
-      <c r="S19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T19" s="4" t="n"/>
-      <c r="U19" s="4" t="n"/>
-      <c r="V19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="28" customHeight="1" s="11">
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="11" t="n"/>
+      <c r="I19" s="11" t="n"/>
+      <c r="J19" s="11" t="n"/>
+      <c r="K19" s="11" t="n"/>
+      <c r="L19" s="11" t="n"/>
+      <c r="M19" s="11" t="n"/>
+      <c r="N19" s="11" t="n"/>
+      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
+      <c r="Q19" s="11" t="n"/>
+      <c r="R19" s="11" t="n"/>
+      <c r="S19" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T19" s="11" t="n"/>
+      <c r="U19" s="11" t="n"/>
+      <c r="V19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Hospitalisation / sortie</t>
@@ -2108,7 +2130,7 @@
       </c>
       <c r="T20" s="5" t="n"/>
       <c r="U20" s="5" t="n"/>
-      <c r="V20" s="4" t="n"/>
+      <c r="V20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -2137,30 +2159,30 @@
         </is>
       </c>
       <c r="F21" s="3" t="n"/>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" s="4" t="n"/>
-      <c r="I21" s="4" t="n"/>
-      <c r="J21" s="4" t="n"/>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="n"/>
-      <c r="M21" s="4" t="n"/>
-      <c r="N21" s="4" t="n"/>
-      <c r="O21" s="4" t="n"/>
-      <c r="P21" s="4" t="n"/>
-      <c r="Q21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R21" s="4" t="n"/>
-      <c r="S21" s="4" t="n"/>
-      <c r="T21" s="4" t="n"/>
-      <c r="U21" s="4" t="n"/>
-      <c r="V21" s="4" t="n"/>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="11" t="n"/>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
+      <c r="Q21" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="n"/>
+      <c r="S21" s="11" t="n"/>
+      <c r="T21" s="11" t="n"/>
+      <c r="U21" s="11" t="n"/>
+      <c r="V21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2189,36 +2211,36 @@
         </is>
       </c>
       <c r="F22" s="3" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="n"/>
-      <c r="M22" s="4" t="n"/>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P22" s="4" t="n"/>
-      <c r="Q22" s="4" t="n"/>
-      <c r="R22" s="4" t="n"/>
-      <c r="S22" s="4" t="n"/>
-      <c r="T22" s="4" t="n"/>
-      <c r="U22" s="4" t="n"/>
-      <c r="V22" s="4" t="n"/>
-    </row>
-    <row r="23" ht="28" customHeight="1" s="11">
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="11" t="n"/>
+      <c r="I22" s="11" t="n"/>
+      <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="n"/>
+      <c r="N22" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P22" s="11" t="n"/>
+      <c r="Q22" s="11" t="n"/>
+      <c r="R22" s="11" t="n"/>
+      <c r="S22" s="11" t="n"/>
+      <c r="T22" s="11" t="n"/>
+      <c r="U22" s="11" t="n"/>
+      <c r="V22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="28.05" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Maintien à domicile</t>
@@ -2268,9 +2290,9 @@
       <c r="S23" s="5" t="n"/>
       <c r="T23" s="5" t="n"/>
       <c r="U23" s="5" t="n"/>
-      <c r="V23" s="4" t="inlineStr">
-        <is>
-          <t>Contacter les services d'aide à domicile du secteur.</t>
+      <c r="V23" s="11" t="inlineStr">
+        <is>
+          <t>Contacter les services d'aide à domicile du secteur : annuaire des [Services d'aide à domicile (SAAD) du Var](https://www.sanitaire-social.com/annuaire-soins-et-aide-a-domicile/services-d-aide-a-domicile-sad/liste-var-83) ou annuaire des [SSIAD du Var](https://www.capgeris.com/ssiad/provence-alpes-cote-d-azur/var/).</t>
         </is>
       </c>
     </row>
@@ -2301,38 +2323,38 @@
         </is>
       </c>
       <c r="F24" s="3" t="n"/>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
-      <c r="I24" s="4" t="n"/>
-      <c r="J24" s="4" t="n"/>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="n"/>
-      <c r="M24" s="4" t="n"/>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P24" s="4" t="n"/>
-      <c r="Q24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R24" s="4" t="n"/>
-      <c r="S24" s="4" t="n"/>
-      <c r="T24" s="4" t="n"/>
-      <c r="U24" s="4" t="n"/>
-      <c r="V24" s="4" t="n"/>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="11" t="n"/>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="11" t="n"/>
+      <c r="N24" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O24" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P24" s="11" t="n"/>
+      <c r="Q24" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="n"/>
+      <c r="S24" s="11" t="n"/>
+      <c r="T24" s="11" t="n"/>
+      <c r="U24" s="11" t="n"/>
+      <c r="V24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2388,7 +2410,7 @@
       <c r="S25" s="5" t="n"/>
       <c r="T25" s="5" t="n"/>
       <c r="U25" s="5" t="n"/>
-      <c r="V25" s="4" t="n"/>
+      <c r="V25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2432,13 +2454,13 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="R26" s="4" t="n"/>
-      <c r="S26" s="4" t="n"/>
-      <c r="T26" s="4" t="n"/>
-      <c r="U26" s="4" t="n"/>
-      <c r="V26" s="4" t="n"/>
-    </row>
-    <row r="27" ht="17.65" customHeight="1" s="11">
+      <c r="R26" s="11" t="n"/>
+      <c r="S26" s="11" t="n"/>
+      <c r="T26" s="11" t="n"/>
+      <c r="U26" s="11" t="n"/>
+      <c r="V26" s="11" t="n"/>
+    </row>
+    <row r="27" ht="17.7" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Maintien à domicile</t>
@@ -2465,34 +2487,34 @@
         </is>
       </c>
       <c r="F27" s="3" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R27" s="4" t="n"/>
-      <c r="S27" s="4" t="n"/>
-      <c r="T27" s="4" t="n"/>
-      <c r="U27" s="4" t="n"/>
-      <c r="V27" s="4" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="11" t="n"/>
+      <c r="I27" s="11" t="n"/>
+      <c r="J27" s="11" t="n"/>
+      <c r="K27" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L27" s="11" t="n"/>
+      <c r="M27" s="11" t="n"/>
+      <c r="N27" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O27" s="11" t="n"/>
+      <c r="P27" s="11" t="n"/>
+      <c r="Q27" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R27" s="11" t="n"/>
+      <c r="S27" s="11" t="n"/>
+      <c r="T27" s="11" t="n"/>
+      <c r="U27" s="11" t="n"/>
+      <c r="V27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2552,9 +2574,9 @@
       <c r="S28" s="5" t="n"/>
       <c r="T28" s="5" t="n"/>
       <c r="U28" s="5" t="n"/>
-      <c r="V28" s="4" t="n"/>
-    </row>
-    <row r="29" ht="17.65" customHeight="1" s="11">
+      <c r="V28" s="11" t="n"/>
+    </row>
+    <row r="29" ht="17.7" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Maintien à domicile</t>
@@ -2581,28 +2603,28 @@
         </is>
       </c>
       <c r="F29" s="3" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="4" t="n"/>
-      <c r="Q29" s="4" t="n"/>
-      <c r="R29" s="4" t="n"/>
-      <c r="S29" s="4" t="n"/>
-      <c r="T29" s="4" t="n"/>
-      <c r="U29" s="4" t="n"/>
-      <c r="V29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="17.65" customHeight="1" s="11">
+      <c r="G29" s="11" t="n"/>
+      <c r="H29" s="11" t="n"/>
+      <c r="I29" s="11" t="n"/>
+      <c r="J29" s="11" t="n"/>
+      <c r="K29" s="11" t="n"/>
+      <c r="L29" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M29" s="11" t="n"/>
+      <c r="N29" s="11" t="n"/>
+      <c r="O29" s="11" t="n"/>
+      <c r="P29" s="11" t="n"/>
+      <c r="Q29" s="11" t="n"/>
+      <c r="R29" s="11" t="n"/>
+      <c r="S29" s="11" t="n"/>
+      <c r="T29" s="11" t="n"/>
+      <c r="U29" s="11" t="n"/>
+      <c r="V29" s="11" t="n"/>
+    </row>
+    <row r="30" ht="17.7" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Maintien à domicile</t>
@@ -2648,9 +2670,9 @@
       <c r="S30" s="5" t="n"/>
       <c r="T30" s="5" t="n"/>
       <c r="U30" s="5" t="n"/>
-      <c r="V30" s="4" t="n"/>
-    </row>
-    <row r="31">
+      <c r="V30" s="11" t="n"/>
+    </row>
+    <row r="31" ht="27.6" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Autonomie / aidants</t>
@@ -2677,28 +2699,28 @@
         </is>
       </c>
       <c r="F31" s="3" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
-      <c r="K31" s="4" t="n"/>
-      <c r="L31" s="4" t="n"/>
-      <c r="M31" s="4" t="n"/>
-      <c r="N31" s="4" t="n"/>
-      <c r="O31" s="4" t="n"/>
-      <c r="P31" s="4" t="n"/>
-      <c r="Q31" s="4" t="n"/>
-      <c r="R31" s="4" t="n"/>
-      <c r="S31" s="4" t="n"/>
-      <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U31" s="4" t="n"/>
-      <c r="V31" s="4" t="inlineStr">
-        <is>
-          <t>Se rapprocher de l'association des aidants.</t>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="n"/>
+      <c r="I31" s="11" t="n"/>
+      <c r="J31" s="11" t="n"/>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
+      <c r="M31" s="11" t="n"/>
+      <c r="N31" s="11" t="n"/>
+      <c r="O31" s="11" t="n"/>
+      <c r="P31" s="11" t="n"/>
+      <c r="Q31" s="11" t="n"/>
+      <c r="R31" s="11" t="n"/>
+      <c r="S31" s="11" t="n"/>
+      <c r="T31" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U31" s="11" t="n"/>
+      <c r="V31" s="11" t="inlineStr">
+        <is>
+          <t>Se rapprocher des [Associations des aidants (Var)](https://maboussoleaidants.fr/mes-solutions/associations-aidants/83) et des plateformes de répit.</t>
         </is>
       </c>
     </row>
@@ -2729,28 +2751,28 @@
         </is>
       </c>
       <c r="F32" s="3" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="n"/>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="n"/>
-      <c r="M32" s="4" t="n"/>
-      <c r="N32" s="4" t="n"/>
-      <c r="O32" s="4" t="n"/>
-      <c r="P32" s="4" t="n"/>
-      <c r="Q32" s="4" t="n"/>
-      <c r="R32" s="4" t="n"/>
-      <c r="S32" s="4" t="n"/>
-      <c r="T32" s="4" t="n"/>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="n"/>
-    </row>
-    <row r="33" ht="28" customHeight="1" s="11">
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="11" t="n"/>
+      <c r="I32" s="11" t="n"/>
+      <c r="J32" s="11" t="n"/>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="11" t="n"/>
+      <c r="M32" s="11" t="n"/>
+      <c r="N32" s="11" t="n"/>
+      <c r="O32" s="11" t="n"/>
+      <c r="P32" s="11" t="n"/>
+      <c r="Q32" s="11" t="n"/>
+      <c r="R32" s="11" t="n"/>
+      <c r="S32" s="11" t="n"/>
+      <c r="T32" s="11" t="n"/>
+      <c r="U32" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V32" s="11" t="n"/>
+    </row>
+    <row r="33" ht="28.05" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Autonomie / aidants</t>
@@ -2808,9 +2830,9 @@
       <c r="S33" s="5" t="n"/>
       <c r="T33" s="5" t="n"/>
       <c r="U33" s="5" t="n"/>
-      <c r="V33" s="4" t="n"/>
-    </row>
-    <row r="34" ht="28" customHeight="1" s="11">
+      <c r="V33" s="11" t="n"/>
+    </row>
+    <row r="34" ht="28.05" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Autonomie / aidants</t>
@@ -2864,9 +2886,9 @@
       <c r="S34" s="5" t="n"/>
       <c r="T34" s="5" t="n"/>
       <c r="U34" s="5" t="n"/>
-      <c r="V34" s="4" t="n"/>
-    </row>
-    <row r="35" ht="28" customHeight="1" s="11">
+      <c r="V34" s="11" t="n"/>
+    </row>
+    <row r="35" ht="28.05" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Autonomie / aidants</t>
@@ -2893,30 +2915,30 @@
         </is>
       </c>
       <c r="F35" s="3" t="n"/>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L35" s="4" t="n"/>
-      <c r="M35" s="4" t="n"/>
-      <c r="N35" s="4" t="n"/>
-      <c r="O35" s="4" t="n"/>
-      <c r="P35" s="4" t="n"/>
-      <c r="Q35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R35" s="4" t="n"/>
-      <c r="S35" s="4" t="n"/>
-      <c r="T35" s="4" t="n"/>
-      <c r="U35" s="4" t="n"/>
-      <c r="V35" s="4" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="11" t="n"/>
+      <c r="I35" s="11" t="n"/>
+      <c r="J35" s="11" t="n"/>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L35" s="11" t="n"/>
+      <c r="M35" s="11" t="n"/>
+      <c r="N35" s="11" t="n"/>
+      <c r="O35" s="11" t="n"/>
+      <c r="P35" s="11" t="n"/>
+      <c r="Q35" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R35" s="11" t="n"/>
+      <c r="S35" s="11" t="n"/>
+      <c r="T35" s="11" t="n"/>
+      <c r="U35" s="11" t="n"/>
+      <c r="V35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2945,34 +2967,34 @@
         </is>
       </c>
       <c r="F36" s="3" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M36" s="4" t="n"/>
-      <c r="N36" s="4" t="n"/>
-      <c r="O36" s="4" t="n"/>
-      <c r="P36" s="4" t="n"/>
-      <c r="Q36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R36" s="4" t="n"/>
-      <c r="S36" s="4" t="n"/>
-      <c r="T36" s="4" t="n"/>
-      <c r="U36" s="4" t="n"/>
-      <c r="V36" s="4" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="11" t="n"/>
+      <c r="I36" s="11" t="n"/>
+      <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M36" s="11" t="n"/>
+      <c r="N36" s="11" t="n"/>
+      <c r="O36" s="11" t="n"/>
+      <c r="P36" s="11" t="n"/>
+      <c r="Q36" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R36" s="11" t="n"/>
+      <c r="S36" s="11" t="n"/>
+      <c r="T36" s="11" t="n"/>
+      <c r="U36" s="11" t="n"/>
+      <c r="V36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3028,9 +3050,9 @@
       <c r="S37" s="5" t="n"/>
       <c r="T37" s="5" t="n"/>
       <c r="U37" s="5" t="n"/>
-      <c r="V37" s="4" t="n"/>
-    </row>
-    <row r="38" ht="28" customHeight="1" s="11">
+      <c r="V37" s="11" t="n"/>
+    </row>
+    <row r="38" ht="28.05" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Autonomie / aidants</t>
@@ -3057,32 +3079,32 @@
         </is>
       </c>
       <c r="F38" s="3" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="n"/>
-      <c r="K38" s="4" t="n"/>
-      <c r="L38" s="4" t="n"/>
-      <c r="M38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N38" s="4" t="n"/>
-      <c r="O38" s="4" t="n"/>
-      <c r="P38" s="4" t="n"/>
-      <c r="Q38" s="4" t="n"/>
-      <c r="R38" s="4" t="n"/>
-      <c r="S38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T38" s="4" t="n"/>
-      <c r="U38" s="4" t="n"/>
-      <c r="V38" s="4" t="inlineStr">
-        <is>
-          <t>S'orienter vers le médecin traitant ou un médecin spécialiste.</t>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="11" t="n"/>
+      <c r="I38" s="11" t="n"/>
+      <c r="J38" s="11" t="n"/>
+      <c r="K38" s="11" t="n"/>
+      <c r="L38" s="11" t="n"/>
+      <c r="M38" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N38" s="11" t="n"/>
+      <c r="O38" s="11" t="n"/>
+      <c r="P38" s="11" t="n"/>
+      <c r="Q38" s="11" t="n"/>
+      <c r="R38" s="11" t="n"/>
+      <c r="S38" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T38" s="11" t="n"/>
+      <c r="U38" s="11" t="n"/>
+      <c r="V38" s="11" t="inlineStr">
+        <is>
+          <t>Orienter vers le médecin traitant ou un médecin spécialiste.</t>
         </is>
       </c>
     </row>
@@ -3113,32 +3135,32 @@
         </is>
       </c>
       <c r="F39" s="3" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
-      <c r="I39" s="4" t="n"/>
-      <c r="J39" s="4" t="n"/>
-      <c r="K39" s="4" t="n"/>
-      <c r="L39" s="4" t="n"/>
-      <c r="M39" s="4" t="n"/>
-      <c r="N39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="n"/>
-      <c r="P39" s="4" t="n"/>
-      <c r="Q39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R39" s="4" t="n"/>
-      <c r="S39" s="4" t="n"/>
-      <c r="T39" s="4" t="n"/>
-      <c r="U39" s="4" t="n"/>
-      <c r="V39" s="4" t="n"/>
-    </row>
-    <row r="40" ht="17.65" customHeight="1" s="11">
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="11" t="n"/>
+      <c r="I39" s="11" t="n"/>
+      <c r="J39" s="11" t="n"/>
+      <c r="K39" s="11" t="n"/>
+      <c r="L39" s="11" t="n"/>
+      <c r="M39" s="11" t="n"/>
+      <c r="N39" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O39" s="11" t="n"/>
+      <c r="P39" s="11" t="n"/>
+      <c r="Q39" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R39" s="11" t="n"/>
+      <c r="S39" s="11" t="n"/>
+      <c r="T39" s="11" t="n"/>
+      <c r="U39" s="11" t="n"/>
+      <c r="V39" s="11" t="n"/>
+    </row>
+    <row r="40" ht="17.7" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3188,9 +3210,9 @@
       <c r="S40" s="5" t="n"/>
       <c r="T40" s="5" t="n"/>
       <c r="U40" s="5" t="n"/>
-      <c r="V40" s="4" t="n"/>
-    </row>
-    <row r="41" ht="17.65" customHeight="1" s="11">
+      <c r="V40" s="11" t="n"/>
+    </row>
+    <row r="41" ht="17.7" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3217,30 +3239,30 @@
         </is>
       </c>
       <c r="F41" s="3" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="n"/>
-      <c r="M41" s="4" t="n"/>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R41" s="4" t="n"/>
-      <c r="S41" s="4" t="n"/>
-      <c r="T41" s="4" t="n"/>
-      <c r="U41" s="4" t="n"/>
-      <c r="V41" s="4" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="11" t="n"/>
+      <c r="J41" s="11" t="n"/>
+      <c r="K41" s="11" t="n"/>
+      <c r="L41" s="11" t="n"/>
+      <c r="M41" s="11" t="n"/>
+      <c r="N41" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O41" s="11" t="n"/>
+      <c r="P41" s="11" t="n"/>
+      <c r="Q41" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R41" s="11" t="n"/>
+      <c r="S41" s="11" t="n"/>
+      <c r="T41" s="11" t="n"/>
+      <c r="U41" s="11" t="n"/>
+      <c r="V41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3292,9 +3314,9 @@
       <c r="S42" s="5" t="n"/>
       <c r="T42" s="5" t="n"/>
       <c r="U42" s="5" t="n"/>
-      <c r="V42" s="4" t="n"/>
-    </row>
-    <row r="43" ht="17.65" customHeight="1" s="11">
+      <c r="V42" s="11" t="n"/>
+    </row>
+    <row r="43" ht="17.7" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3321,32 +3343,32 @@
         </is>
       </c>
       <c r="F43" s="3" t="n"/>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-      <c r="L43" s="4" t="n"/>
-      <c r="M43" s="4" t="n"/>
-      <c r="N43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
-      <c r="Q43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R43" s="4" t="n"/>
-      <c r="S43" s="4" t="n"/>
-      <c r="T43" s="4" t="n"/>
-      <c r="U43" s="4" t="n"/>
-      <c r="V43" s="4" t="n"/>
-    </row>
-    <row r="44" ht="28" customHeight="1" s="11">
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="11" t="n"/>
+      <c r="J43" s="11" t="n"/>
+      <c r="K43" s="11" t="n"/>
+      <c r="L43" s="11" t="n"/>
+      <c r="M43" s="11" t="n"/>
+      <c r="N43" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O43" s="11" t="n"/>
+      <c r="P43" s="11" t="n"/>
+      <c r="Q43" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R43" s="11" t="n"/>
+      <c r="S43" s="11" t="n"/>
+      <c r="T43" s="11" t="n"/>
+      <c r="U43" s="11" t="n"/>
+      <c r="V43" s="11" t="n"/>
+    </row>
+    <row r="44" ht="28.05" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3400,9 +3422,9 @@
       <c r="S44" s="5" t="n"/>
       <c r="T44" s="5" t="n"/>
       <c r="U44" s="5" t="n"/>
-      <c r="V44" s="4" t="n"/>
-    </row>
-    <row r="45" ht="17.65" customHeight="1" s="11">
+      <c r="V44" s="11" t="n"/>
+    </row>
+    <row r="45" ht="17.7" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3452,9 +3474,9 @@
       <c r="S45" s="5" t="n"/>
       <c r="T45" s="5" t="n"/>
       <c r="U45" s="5" t="n"/>
-      <c r="V45" s="4" t="n"/>
-    </row>
-    <row r="46" ht="17.65" customHeight="1" s="11">
+      <c r="V45" s="11" t="n"/>
+    </row>
+    <row r="46" ht="17.7" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3481,36 +3503,36 @@
         </is>
       </c>
       <c r="F46" s="3" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
-      <c r="K46" s="4" t="n"/>
-      <c r="L46" s="4" t="n"/>
-      <c r="M46" s="4" t="n"/>
-      <c r="N46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P46" s="4" t="n"/>
-      <c r="Q46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R46" s="4" t="n"/>
-      <c r="S46" s="4" t="n"/>
-      <c r="T46" s="4" t="n"/>
-      <c r="U46" s="4" t="n"/>
-      <c r="V46" s="4" t="n"/>
-    </row>
-    <row r="47" ht="17.65" customHeight="1" s="11">
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="11" t="n"/>
+      <c r="I46" s="11" t="n"/>
+      <c r="J46" s="11" t="n"/>
+      <c r="K46" s="11" t="n"/>
+      <c r="L46" s="11" t="n"/>
+      <c r="M46" s="11" t="n"/>
+      <c r="N46" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O46" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P46" s="11" t="n"/>
+      <c r="Q46" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R46" s="11" t="n"/>
+      <c r="S46" s="11" t="n"/>
+      <c r="T46" s="11" t="n"/>
+      <c r="U46" s="11" t="n"/>
+      <c r="V46" s="11" t="n"/>
+    </row>
+    <row r="47" ht="17.7" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3544,7 +3566,7 @@
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="5" t="n"/>
       <c r="M47" s="5" t="n"/>
-      <c r="N47" s="4" t="inlineStr">
+      <c r="N47" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3555,7 +3577,7 @@
         </is>
       </c>
       <c r="P47" s="5" t="n"/>
-      <c r="Q47" s="4" t="inlineStr">
+      <c r="Q47" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3564,7 +3586,7 @@
       <c r="S47" s="5" t="n"/>
       <c r="T47" s="5" t="n"/>
       <c r="U47" s="5" t="n"/>
-      <c r="V47" s="4" t="n"/>
+      <c r="V47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3600,7 +3622,7 @@
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="5" t="n"/>
       <c r="M48" s="5" t="n"/>
-      <c r="N48" s="4" t="inlineStr">
+      <c r="N48" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3611,7 +3633,7 @@
         </is>
       </c>
       <c r="P48" s="5" t="n"/>
-      <c r="Q48" s="4" t="inlineStr">
+      <c r="Q48" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3620,7 +3642,7 @@
       <c r="S48" s="5" t="n"/>
       <c r="T48" s="5" t="n"/>
       <c r="U48" s="5" t="n"/>
-      <c r="V48" s="4" t="n"/>
+      <c r="V48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -3649,32 +3671,32 @@
         </is>
       </c>
       <c r="F49" s="3" t="n"/>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
-      <c r="J49" s="4" t="n"/>
-      <c r="K49" s="4" t="n"/>
-      <c r="L49" s="4" t="n"/>
-      <c r="M49" s="4" t="n"/>
-      <c r="N49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O49" s="4" t="n"/>
-      <c r="P49" s="4" t="n"/>
-      <c r="Q49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R49" s="4" t="n"/>
-      <c r="S49" s="4" t="n"/>
-      <c r="T49" s="4" t="n"/>
-      <c r="U49" s="4" t="n"/>
-      <c r="V49" s="4" t="n"/>
-    </row>
-    <row r="50" ht="28" customHeight="1" s="11">
+      <c r="G49" s="11" t="n"/>
+      <c r="H49" s="11" t="n"/>
+      <c r="I49" s="11" t="n"/>
+      <c r="J49" s="11" t="n"/>
+      <c r="K49" s="11" t="n"/>
+      <c r="L49" s="11" t="n"/>
+      <c r="M49" s="11" t="n"/>
+      <c r="N49" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O49" s="11" t="n"/>
+      <c r="P49" s="11" t="n"/>
+      <c r="Q49" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R49" s="11" t="n"/>
+      <c r="S49" s="11" t="n"/>
+      <c r="T49" s="11" t="n"/>
+      <c r="U49" s="11" t="n"/>
+      <c r="V49" s="11" t="n"/>
+    </row>
+    <row r="50" ht="28.05" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3708,14 +3730,14 @@
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="5" t="n"/>
       <c r="M50" s="5" t="n"/>
-      <c r="N50" s="4" t="inlineStr">
+      <c r="N50" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="5" t="n"/>
-      <c r="Q50" s="4" t="inlineStr">
+      <c r="Q50" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3724,9 +3746,9 @@
       <c r="S50" s="5" t="n"/>
       <c r="T50" s="5" t="n"/>
       <c r="U50" s="5" t="n"/>
-      <c r="V50" s="4" t="n"/>
-    </row>
-    <row r="51" ht="28" customHeight="1" s="11">
+      <c r="V50" s="11" t="n"/>
+    </row>
+    <row r="51" ht="28.05" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3753,40 +3775,40 @@
         </is>
       </c>
       <c r="F51" s="3" t="n"/>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="n"/>
-      <c r="L51" s="4" t="n"/>
-      <c r="M51" s="4" t="n"/>
-      <c r="N51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P51" s="4" t="n"/>
-      <c r="Q51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R51" s="4" t="n"/>
-      <c r="S51" s="4" t="n"/>
-      <c r="T51" s="4" t="n"/>
-      <c r="U51" s="4" t="n"/>
-      <c r="V51" s="4" t="n"/>
-    </row>
-    <row r="52" ht="17.65" customHeight="1" s="11">
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="n"/>
+      <c r="I51" s="11" t="n"/>
+      <c r="J51" s="11" t="n"/>
+      <c r="K51" s="11" t="n"/>
+      <c r="L51" s="11" t="n"/>
+      <c r="M51" s="11" t="n"/>
+      <c r="N51" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O51" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P51" s="11" t="n"/>
+      <c r="Q51" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R51" s="11" t="n"/>
+      <c r="S51" s="11" t="n"/>
+      <c r="T51" s="11" t="n"/>
+      <c r="U51" s="11" t="n"/>
+      <c r="V51" s="11" t="n"/>
+    </row>
+    <row r="52" ht="17.7" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3813,34 +3835,34 @@
         </is>
       </c>
       <c r="F52" s="3" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
-      <c r="K52" s="4" t="n"/>
-      <c r="L52" s="4" t="n"/>
-      <c r="M52" s="4" t="n"/>
-      <c r="N52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P52" s="4" t="n"/>
-      <c r="Q52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R52" s="4" t="n"/>
-      <c r="S52" s="4" t="n"/>
-      <c r="T52" s="4" t="n"/>
-      <c r="U52" s="4" t="n"/>
-      <c r="V52" s="4" t="n"/>
+      <c r="G52" s="11" t="n"/>
+      <c r="H52" s="11" t="n"/>
+      <c r="I52" s="11" t="n"/>
+      <c r="J52" s="11" t="n"/>
+      <c r="K52" s="11" t="n"/>
+      <c r="L52" s="11" t="n"/>
+      <c r="M52" s="11" t="n"/>
+      <c r="N52" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O52" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P52" s="11" t="n"/>
+      <c r="Q52" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R52" s="11" t="n"/>
+      <c r="S52" s="11" t="n"/>
+      <c r="T52" s="11" t="n"/>
+      <c r="U52" s="11" t="n"/>
+      <c r="V52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3876,7 +3898,7 @@
       <c r="K53" s="5" t="n"/>
       <c r="L53" s="5" t="n"/>
       <c r="M53" s="5" t="n"/>
-      <c r="N53" s="4" t="inlineStr">
+      <c r="N53" s="11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3896,9 +3918,9 @@
       <c r="S53" s="5" t="n"/>
       <c r="T53" s="5" t="n"/>
       <c r="U53" s="5" t="n"/>
-      <c r="V53" s="4" t="n"/>
-    </row>
-    <row r="54" ht="17.65" customHeight="1" s="11">
+      <c r="V53" s="11" t="n"/>
+    </row>
+    <row r="54" ht="17.7" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3925,32 +3947,32 @@
         </is>
       </c>
       <c r="F54" s="3" t="n"/>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-      <c r="K54" s="4" t="n"/>
-      <c r="L54" s="4" t="n"/>
-      <c r="M54" s="4" t="n"/>
-      <c r="N54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O54" s="4" t="n"/>
-      <c r="P54" s="4" t="n"/>
-      <c r="Q54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R54" s="4" t="n"/>
-      <c r="S54" s="4" t="n"/>
-      <c r="T54" s="4" t="n"/>
-      <c r="U54" s="4" t="n"/>
-      <c r="V54" s="4" t="n"/>
-    </row>
-    <row r="55" ht="17.65" customHeight="1" s="11">
+      <c r="G54" s="11" t="n"/>
+      <c r="H54" s="11" t="n"/>
+      <c r="I54" s="11" t="n"/>
+      <c r="J54" s="11" t="n"/>
+      <c r="K54" s="11" t="n"/>
+      <c r="L54" s="11" t="n"/>
+      <c r="M54" s="11" t="n"/>
+      <c r="N54" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O54" s="11" t="n"/>
+      <c r="P54" s="11" t="n"/>
+      <c r="Q54" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R54" s="11" t="n"/>
+      <c r="S54" s="11" t="n"/>
+      <c r="T54" s="11" t="n"/>
+      <c r="U54" s="11" t="n"/>
+      <c r="V54" s="11" t="n"/>
+    </row>
+    <row r="55" ht="17.7" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -3977,28 +3999,28 @@
         </is>
       </c>
       <c r="F55" s="3" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-      <c r="K55" s="4" t="n"/>
-      <c r="L55" s="4" t="n"/>
-      <c r="M55" s="4" t="n"/>
-      <c r="N55" s="4" t="n"/>
-      <c r="O55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P55" s="4" t="n"/>
-      <c r="Q55" s="4" t="n"/>
-      <c r="R55" s="4" t="n"/>
-      <c r="S55" s="4" t="n"/>
-      <c r="T55" s="4" t="n"/>
-      <c r="U55" s="4" t="n"/>
-      <c r="V55" s="4" t="n"/>
-    </row>
-    <row r="56" ht="28" customHeight="1" s="11">
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
+      <c r="I55" s="11" t="n"/>
+      <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
+      <c r="M55" s="11" t="n"/>
+      <c r="N55" s="11" t="n"/>
+      <c r="O55" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P55" s="11" t="n"/>
+      <c r="Q55" s="11" t="n"/>
+      <c r="R55" s="11" t="n"/>
+      <c r="S55" s="11" t="n"/>
+      <c r="T55" s="11" t="n"/>
+      <c r="U55" s="11" t="n"/>
+      <c r="V55" s="11" t="n"/>
+    </row>
+    <row r="56" ht="28.05" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Social / droits / budget</t>
@@ -4031,7 +4053,7 @@
       <c r="J56" s="9" t="n"/>
       <c r="K56" s="9" t="n"/>
       <c r="L56" s="9" t="n"/>
-      <c r="M56" s="4" t="n"/>
+      <c r="M56" s="11" t="n"/>
       <c r="N56" s="9" t="inlineStr">
         <is>
           <t>✓</t>
@@ -4048,13 +4070,13 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="R56" s="4" t="n"/>
-      <c r="S56" s="4" t="n"/>
-      <c r="T56" s="4" t="n"/>
-      <c r="U56" s="4" t="n"/>
-      <c r="V56" s="4" t="n"/>
-    </row>
-    <row r="57" ht="42" customHeight="1" s="11">
+      <c r="R56" s="11" t="n"/>
+      <c r="S56" s="11" t="n"/>
+      <c r="T56" s="11" t="n"/>
+      <c r="U56" s="11" t="n"/>
+      <c r="V56" s="11" t="n"/>
+    </row>
+    <row r="57" ht="42" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
           <t>Logement / habitat</t>
@@ -4087,7 +4109,7 @@
       <c r="J57" s="10" t="n"/>
       <c r="K57" s="10" t="n"/>
       <c r="L57" s="10" t="n"/>
-      <c r="M57" s="4" t="n"/>
+      <c r="M57" s="11" t="n"/>
       <c r="N57" s="9" t="n"/>
       <c r="O57" s="10" t="n"/>
       <c r="P57" s="10" t="inlineStr">
@@ -4096,17 +4118,17 @@
         </is>
       </c>
       <c r="Q57" s="10" t="n"/>
-      <c r="R57" s="4" t="n"/>
-      <c r="S57" s="4" t="n"/>
-      <c r="T57" s="4" t="n"/>
-      <c r="U57" s="4" t="n"/>
-      <c r="V57" s="4" t="inlineStr">
-        <is>
-          <t>Faire appel à des sociétés de nettoyage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
+      <c r="R57" s="11" t="n"/>
+      <c r="S57" s="11" t="n"/>
+      <c r="T57" s="11" t="n"/>
+      <c r="U57" s="11" t="n"/>
+      <c r="V57" s="11" t="inlineStr">
+        <is>
+          <t>Faire appel à des sociétés spécialisées : consulter l'annuaire des [Entreprises de nettoyage dans le Var](https://www.societe-de-nettoyage.net/entreprise_localisation/toutes-les-regions/paca-provence-alpes-cote-dazur/var/).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="69" customHeight="1">
       <c r="A58" t="inlineStr">
         <is>
           <t>Santé / Addictions</t>
@@ -4122,13 +4144,17 @@
           <t>addiction, alcool, drogue, substance, dependance, addictologie, arcasud</t>
         </is>
       </c>
-      <c r="V58" t="inlineStr">
+      <c r="R58" s="11" t="n"/>
+      <c r="S58" s="11" t="n"/>
+      <c r="T58" s="11" t="n"/>
+      <c r="U58" s="11" t="n"/>
+      <c r="V58" s="11" t="inlineStr">
         <is>
           <t>Se rapprocher d'ARCA Sud ([www.arca-sud.fr](https://www.arca-sud.fr/)) pour tout ce qui concerne la prise en charge des addictions (alcool, drogues, dépendances).</t>
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="124.2" customHeight="1">
       <c r="A59" t="inlineStr">
         <is>
           <t>Social / Droits / Protection</t>
@@ -4144,23 +4170,27 @@
           <t>tutelle, curatelle, protection_juridique, sauvegarde_de_justice, autonomie_decisionnelle, mandataire, mandataire_judiciaire, mjpm, sous_tutelle, sous_curatelle, habilitation_familiale, incapa, incapacite, decisionnelle, tribunal_de_proximite, juge_des_tutelles, gestion_comptes</t>
         </is>
       </c>
-      <c r="V59" t="inlineStr">
+      <c r="R59" s="11" t="n"/>
+      <c r="S59" s="11" t="n"/>
+      <c r="T59" s="11" t="n"/>
+      <c r="U59" s="11" t="n"/>
+      <c r="V59" s="11" t="inlineStr">
         <is>
           <t>Envisager une mesure de protection juridique (tutelle, curatelle, sauvegarde de justice) auprès du tribunal de proximité. Retrouvez plus d'informations sur la fiche [Mesures de protection – DAC Var Ouest](https://dac-varouest.fr/index.php/ressources/minformer/mesures-de-protection/).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:U57">
+  <conditionalFormatting sqref="G2:U59">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>G2="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E2:F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"POLICE,CEV,SERVICE_SOCIAL_HOPITAL,CPTS,CLIC,CRT,DAC,UTS,CCAS,COMPAGNONS_BATISSEURS,PSCG_SS_APA,À valider"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Oui,Non,À valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>